<commit_message>
bugfix wrong times and chatnames
</commit_message>
<xml_diff>
--- a/src/lib/assets/data/004FELI-06_database.xlsx
+++ b/src/lib/assets/data/004FELI-06_database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jas/Documents/01_Uni/Doktorat/Dissertation/Datenanalyse/analysis_tables/01_Databank_tables/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Videos\TiT-visualizations\src\lib\assets\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D412B4B8-89A9-C64A-9B08-76EE587EC4AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2A2A1FD-38BC-4589-8E0B-A4235CDF4D1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="68800" windowHeight="27060" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="18345" yWindow="840" windowWidth="27060" windowHeight="20880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Messages" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="689" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="689" uniqueCount="182">
   <si>
     <t>recording_id</t>
   </si>
@@ -98,9 +98,6 @@
   </si>
   <si>
     <t>André Taber</t>
-  </si>
-  <si>
-    <t>felicitas Albrecht</t>
   </si>
   <si>
     <t>Würde spazieren. Halber Tag frei unter der Woche klingt gut</t>
@@ -950,7 +947,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L76"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -963,7 +960,7 @@
     <col min="12" max="12" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1001,7 +998,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -1052,7 +1049,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -1066,7 +1063,7 @@
         <v>20</v>
       </c>
       <c r="E3" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="F3" t="s">
         <v>16</v>
@@ -1100,10 +1097,10 @@
         <v>18</v>
       </c>
       <c r="L3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1120,10 +1117,10 @@
         <v>20</v>
       </c>
       <c r="F4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" t="s">
         <v>23</v>
-      </c>
-      <c r="G4" t="s">
-        <v>24</v>
       </c>
       <c r="H4" t="str">
         <f>IF(
@@ -1151,10 +1148,10 @@
         <v>18</v>
       </c>
       <c r="L4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -1171,10 +1168,10 @@
         <v>14</v>
       </c>
       <c r="F5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H5" t="str">
         <f>IF(
@@ -1196,18 +1193,18 @@
         <v>08:19:45</v>
       </c>
       <c r="J5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K5" t="s">
+        <v>18</v>
+      </c>
+      <c r="L5" t="s">
         <v>27</v>
       </c>
-      <c r="K5" t="s">
-        <v>18</v>
-      </c>
-      <c r="L5" t="s">
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>29</v>
       </c>
       <c r="B6" t="s">
         <v>13</v>
@@ -1222,7 +1219,7 @@
         <v>14</v>
       </c>
       <c r="F6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H6" s="1">
         <v>0.34722222222222221</v>
@@ -1234,12 +1231,12 @@
         <v>18</v>
       </c>
       <c r="L6" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B7" t="s">
         <v>13</v>
@@ -1285,12 +1282,12 @@
         <v>18</v>
       </c>
       <c r="L7" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B8" t="s">
         <v>13</v>
@@ -1305,10 +1302,10 @@
         <v>14</v>
       </c>
       <c r="F8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H8" t="str">
         <f>IF(
@@ -1336,12 +1333,12 @@
         <v>18</v>
       </c>
       <c r="L8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>33</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>34</v>
       </c>
       <c r="B9" t="s">
         <v>13</v>
@@ -1350,7 +1347,7 @@
         <v>8</v>
       </c>
       <c r="D9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E9" t="s">
         <v>15</v>
@@ -1387,12 +1384,12 @@
         <v>18</v>
       </c>
       <c r="L9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B10" t="s">
         <v>13</v>
@@ -1404,13 +1401,13 @@
         <v>15</v>
       </c>
       <c r="E10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H10" t="str">
         <f>IF(
@@ -1438,12 +1435,12 @@
         <v>18</v>
       </c>
       <c r="L10" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B11" t="s">
         <v>13</v>
@@ -1489,12 +1486,12 @@
         <v>18</v>
       </c>
       <c r="L11" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B12" t="s">
         <v>13</v>
@@ -1540,12 +1537,12 @@
         <v>18</v>
       </c>
       <c r="L12" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B13" t="s">
         <v>13</v>
@@ -1591,12 +1588,12 @@
         <v>18</v>
       </c>
       <c r="L13" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B14" t="s">
         <v>13</v>
@@ -1611,10 +1608,10 @@
         <v>20</v>
       </c>
       <c r="F14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H14" t="str">
         <f>IF(
@@ -1642,12 +1639,12 @@
         <v>18</v>
       </c>
       <c r="L14" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B15" t="s">
         <v>13</v>
@@ -1662,10 +1659,10 @@
         <v>20</v>
       </c>
       <c r="F15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H15" t="str">
         <f>IF(
@@ -1693,21 +1690,21 @@
         <v>18</v>
       </c>
       <c r="L15" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" t="s">
+        <v>13</v>
+      </c>
+      <c r="C16">
+        <v>15</v>
+      </c>
+      <c r="D16" t="s">
         <v>34</v>
-      </c>
-      <c r="B16" t="s">
-        <v>13</v>
-      </c>
-      <c r="C16">
-        <v>15</v>
-      </c>
-      <c r="D16" t="s">
-        <v>35</v>
       </c>
       <c r="E16" t="s">
         <v>15</v>
@@ -1744,12 +1741,12 @@
         <v>18</v>
       </c>
       <c r="L16" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B17" t="s">
         <v>13</v>
@@ -1761,13 +1758,13 @@
         <v>15</v>
       </c>
       <c r="E17" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F17" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H17" t="str">
         <f>IF(
@@ -1795,13 +1792,13 @@
         <v>18</v>
       </c>
       <c r="L17" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>49</v>
-      </c>
       <c r="B18" t="s">
         <v>13</v>
       </c>
@@ -1809,7 +1806,7 @@
         <v>17</v>
       </c>
       <c r="D18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E18" t="s">
         <v>15</v>
@@ -1846,30 +1843,30 @@
         <v>18</v>
       </c>
       <c r="L18" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19">
+        <v>18</v>
+      </c>
+      <c r="D19" t="s">
+        <v>15</v>
+      </c>
+      <c r="E19" t="s">
+        <v>34</v>
+      </c>
+      <c r="F19" t="s">
+        <v>22</v>
+      </c>
+      <c r="G19" t="s">
         <v>50</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>49</v>
-      </c>
-      <c r="B19" t="s">
-        <v>13</v>
-      </c>
-      <c r="C19">
-        <v>18</v>
-      </c>
-      <c r="D19" t="s">
-        <v>15</v>
-      </c>
-      <c r="E19" t="s">
-        <v>35</v>
-      </c>
-      <c r="F19" t="s">
-        <v>23</v>
-      </c>
-      <c r="G19" t="s">
-        <v>51</v>
       </c>
       <c r="H19" t="str">
         <f>IF(
@@ -1897,12 +1894,12 @@
         <v>18</v>
       </c>
       <c r="L19" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B20" t="s">
         <v>13</v>
@@ -1914,13 +1911,13 @@
         <v>15</v>
       </c>
       <c r="E20" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F20" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G20" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H20" t="str">
         <f>IF(
@@ -1948,12 +1945,12 @@
         <v>18</v>
       </c>
       <c r="L20" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>54</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>55</v>
       </c>
       <c r="B21" t="s">
         <v>13</v>
@@ -1962,7 +1959,7 @@
         <v>20</v>
       </c>
       <c r="D21" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E21" t="s">
         <v>15</v>
@@ -1993,18 +1990,18 @@
         <v>0.37708333333333333</v>
       </c>
       <c r="J21" t="s">
+        <v>55</v>
+      </c>
+      <c r="K21" t="s">
         <v>56</v>
       </c>
-      <c r="K21" t="s">
+      <c r="L21" t="s">
         <v>57</v>
       </c>
-      <c r="L21" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B22" t="s">
         <v>13</v>
@@ -2016,13 +2013,13 @@
         <v>15</v>
       </c>
       <c r="E22" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G22" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H22" t="str">
         <f>IF(
@@ -2044,18 +2041,18 @@
         <v>09:18:06</v>
       </c>
       <c r="J22" t="s">
+        <v>59</v>
+      </c>
+      <c r="K22" t="s">
+        <v>56</v>
+      </c>
+      <c r="L22" t="s">
         <v>60</v>
       </c>
-      <c r="K22" t="s">
-        <v>57</v>
-      </c>
-      <c r="L22" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B23" t="s">
         <v>13</v>
@@ -2101,12 +2098,12 @@
         <v>18</v>
       </c>
       <c r="L23" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B24" t="s">
         <v>13</v>
@@ -2118,7 +2115,7 @@
         <v>20</v>
       </c>
       <c r="E24" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F24" t="s">
         <v>16</v>
@@ -2146,21 +2143,21 @@
         <v>0.38819444444444451</v>
       </c>
       <c r="J24" t="s">
+        <v>63</v>
+      </c>
+      <c r="K24" t="s">
+        <v>18</v>
+      </c>
+      <c r="L24" t="s">
         <v>64</v>
       </c>
-      <c r="K24" t="s">
-        <v>18</v>
-      </c>
-      <c r="L24" t="s">
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
+      <c r="B25" t="s">
         <v>66</v>
-      </c>
-      <c r="B25" t="s">
-        <v>67</v>
       </c>
       <c r="C25">
         <v>24</v>
@@ -2169,13 +2166,13 @@
         <v>15</v>
       </c>
       <c r="E25" t="s">
+        <v>67</v>
+      </c>
+      <c r="F25" t="s">
+        <v>22</v>
+      </c>
+      <c r="G25" t="s">
         <v>68</v>
-      </c>
-      <c r="F25" t="s">
-        <v>23</v>
-      </c>
-      <c r="G25" t="s">
-        <v>69</v>
       </c>
       <c r="H25" t="str">
         <f>IF(
@@ -2197,18 +2194,18 @@
         <v>09:28:12</v>
       </c>
       <c r="J25" t="s">
+        <v>69</v>
+      </c>
+      <c r="K25" t="s">
+        <v>18</v>
+      </c>
+      <c r="L25" t="s">
         <v>70</v>
       </c>
-      <c r="K25" t="s">
-        <v>18</v>
-      </c>
-      <c r="L25" t="s">
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>71</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
-        <v>72</v>
       </c>
       <c r="B26" t="s">
         <v>13</v>
@@ -2254,12 +2251,12 @@
         <v>18</v>
       </c>
       <c r="L26" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B27" t="s">
         <v>13</v>
@@ -2274,10 +2271,10 @@
         <v>20</v>
       </c>
       <c r="F27" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G27" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H27" t="str">
         <f>IF(
@@ -2305,12 +2302,12 @@
         <v>18</v>
       </c>
       <c r="L27" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>75</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
-        <v>76</v>
       </c>
       <c r="B28" t="s">
         <v>13</v>
@@ -2356,12 +2353,12 @@
         <v>18</v>
       </c>
       <c r="L28" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B29" t="s">
         <v>13</v>
@@ -2376,10 +2373,10 @@
         <v>20</v>
       </c>
       <c r="F29" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G29" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H29" t="str">
         <f>IF(
@@ -2401,18 +2398,18 @@
         <v>11:50:10</v>
       </c>
       <c r="J29" t="s">
+        <v>78</v>
+      </c>
+      <c r="K29" t="s">
+        <v>56</v>
+      </c>
+      <c r="L29" t="s">
         <v>79</v>
       </c>
-      <c r="K29" t="s">
-        <v>57</v>
-      </c>
-      <c r="L29" t="s">
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>80</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
-        <v>81</v>
       </c>
       <c r="B30" t="s">
         <v>13</v>
@@ -2427,21 +2424,21 @@
         <v>20</v>
       </c>
       <c r="F30" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H30" s="1">
         <v>0.51388888888888884</v>
       </c>
       <c r="J30" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="K30" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B31" t="s">
         <v>13</v>
@@ -2478,15 +2475,15 @@
         <v/>
       </c>
       <c r="J31" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="K31" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B32" t="s">
         <v>13</v>
@@ -2523,18 +2520,18 @@
         <v/>
       </c>
       <c r="J32" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K32" t="s">
         <v>18</v>
       </c>
       <c r="L32" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B33" t="s">
         <v>13</v>
@@ -2577,12 +2574,12 @@
         <v>18</v>
       </c>
       <c r="L33" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B34" t="s">
         <v>13</v>
@@ -2597,10 +2594,10 @@
         <v>20</v>
       </c>
       <c r="F34" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G34" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H34" t="str">
         <f>IF(
@@ -2625,15 +2622,15 @@
         <v>17</v>
       </c>
       <c r="K34" t="s">
+        <v>85</v>
+      </c>
+      <c r="L34" t="s">
         <v>86</v>
       </c>
-      <c r="L34" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B35" t="s">
         <v>13</v>
@@ -2648,10 +2645,10 @@
         <v>20</v>
       </c>
       <c r="F35" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G35" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H35" t="str">
         <f>IF(
@@ -2679,12 +2676,12 @@
         <v>18</v>
       </c>
       <c r="L35" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>89</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>90</v>
       </c>
       <c r="B36" t="s">
         <v>13</v>
@@ -2730,12 +2727,12 @@
         <v>18</v>
       </c>
       <c r="L36" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B37" t="s">
         <v>13</v>
@@ -2781,12 +2778,12 @@
         <v>18</v>
       </c>
       <c r="L37" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B38" t="s">
         <v>13</v>
@@ -2801,10 +2798,10 @@
         <v>20</v>
       </c>
       <c r="F38" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G38" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H38" t="str">
         <f>IF(
@@ -2832,12 +2829,12 @@
         <v>18</v>
       </c>
       <c r="L38" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B39" t="s">
         <v>13</v>
@@ -2877,18 +2874,18 @@
         <v>0.64027777777777772</v>
       </c>
       <c r="J39" t="s">
+        <v>94</v>
+      </c>
+      <c r="K39" t="s">
+        <v>18</v>
+      </c>
+      <c r="L39" t="s">
         <v>95</v>
       </c>
-      <c r="K39" t="s">
-        <v>18</v>
-      </c>
-      <c r="L39" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B40" t="s">
         <v>13</v>
@@ -2903,10 +2900,10 @@
         <v>20</v>
       </c>
       <c r="F40" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G40" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H40" t="str">
         <f>IF(
@@ -2928,18 +2925,18 @@
         <v>15:22:12</v>
       </c>
       <c r="J40" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="K40" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="L40" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B41" t="s">
         <v>13</v>
@@ -2985,12 +2982,12 @@
         <v>18</v>
       </c>
       <c r="L41" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B42" t="s">
         <v>13</v>
@@ -3005,10 +3002,10 @@
         <v>20</v>
       </c>
       <c r="F42" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G42" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H42" t="str">
         <f>IF(
@@ -3036,12 +3033,12 @@
         <v>18</v>
       </c>
       <c r="L42" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B43" t="s">
         <v>13</v>
@@ -3056,10 +3053,10 @@
         <v>20</v>
       </c>
       <c r="F43" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G43" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H43" t="str">
         <f>IF(
@@ -3087,12 +3084,12 @@
         <v>18</v>
       </c>
       <c r="L43" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>103</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>104</v>
       </c>
       <c r="B44" t="s">
         <v>13</v>
@@ -3107,10 +3104,10 @@
         <v>20</v>
       </c>
       <c r="F44" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G44" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H44" t="str">
         <f>IF(
@@ -3132,18 +3129,18 @@
         <v>15:24:05</v>
       </c>
       <c r="J44" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K44" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="L44" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B45" t="s">
         <v>13</v>
@@ -3158,10 +3155,10 @@
         <v>20</v>
       </c>
       <c r="F45" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G45" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H45" t="str">
         <f>IF(
@@ -3189,12 +3186,12 @@
         <v>18</v>
       </c>
       <c r="L45" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>108</v>
-      </c>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
-        <v>109</v>
       </c>
       <c r="B46" t="s">
         <v>13</v>
@@ -3203,7 +3200,7 @@
         <v>45</v>
       </c>
       <c r="D46" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E46" t="s">
         <v>15</v>
@@ -3215,18 +3212,18 @@
         <v>0.52361111111111114</v>
       </c>
       <c r="J46" t="s">
+        <v>109</v>
+      </c>
+      <c r="K46" t="s">
+        <v>18</v>
+      </c>
+      <c r="L46" t="s">
         <v>110</v>
       </c>
-      <c r="K46" t="s">
-        <v>18</v>
-      </c>
-      <c r="L46" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B47" t="s">
         <v>13</v>
@@ -3238,10 +3235,10 @@
         <v>15</v>
       </c>
       <c r="E47" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F47" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I47" s="1">
         <v>0.52430555555555558</v>
@@ -3253,12 +3250,12 @@
         <v>18</v>
       </c>
       <c r="L47" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
         <v>112</v>
-      </c>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
-        <v>113</v>
       </c>
       <c r="B48" t="s">
         <v>13</v>
@@ -3304,12 +3301,12 @@
         <v>18</v>
       </c>
       <c r="L48" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B49" t="s">
         <v>13</v>
@@ -3355,12 +3352,12 @@
         <v>18</v>
       </c>
       <c r="L49" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B50" t="s">
         <v>13</v>
@@ -3375,10 +3372,10 @@
         <v>20</v>
       </c>
       <c r="F50" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G50" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H50" t="str">
         <f>IF(
@@ -3400,18 +3397,18 @@
         <v>15:52:01</v>
       </c>
       <c r="J50" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K50" t="s">
         <v>18</v>
       </c>
       <c r="L50" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B51" t="s">
         <v>13</v>
@@ -3426,10 +3423,10 @@
         <v>20</v>
       </c>
       <c r="F51" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G51" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H51" t="str">
         <f>IF(
@@ -3457,15 +3454,15 @@
         <v>18</v>
       </c>
       <c r="L51" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
-        <v>120</v>
-      </c>
       <c r="B52" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C52">
         <v>51</v>
@@ -3502,21 +3499,21 @@
         <v>2.8472222222222222E-2</v>
       </c>
       <c r="J52" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K52" t="s">
         <v>18</v>
       </c>
       <c r="L52" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B53" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C53">
         <v>52</v>
@@ -3553,21 +3550,21 @@
         <v>0</v>
       </c>
       <c r="J53" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K53" t="s">
         <v>18</v>
       </c>
       <c r="L53" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B54" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C54">
         <v>53</v>
@@ -3601,21 +3598,21 @@
         <v/>
       </c>
       <c r="I54" t="s">
+        <v>122</v>
+      </c>
+      <c r="J54" t="s">
+        <v>69</v>
+      </c>
+      <c r="K54" t="s">
+        <v>18</v>
+      </c>
+      <c r="L54" t="s">
         <v>123</v>
       </c>
-      <c r="J54" t="s">
-        <v>70</v>
-      </c>
-      <c r="K54" t="s">
-        <v>18</v>
-      </c>
-      <c r="L54" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B55" t="s">
         <v>13</v>
@@ -3630,10 +3627,10 @@
         <v>14</v>
       </c>
       <c r="F55" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G55" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H55" t="str">
         <f>IF(
@@ -3661,12 +3658,12 @@
         <v>18</v>
       </c>
       <c r="L55" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B56" t="s">
         <v>13</v>
@@ -3681,10 +3678,10 @@
         <v>14</v>
       </c>
       <c r="F56" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G56" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H56" t="str">
         <f>IF(
@@ -3706,18 +3703,18 @@
         <v>19:02:05</v>
       </c>
       <c r="J56" t="s">
+        <v>127</v>
+      </c>
+      <c r="K56" t="s">
+        <v>18</v>
+      </c>
+      <c r="L56" t="s">
         <v>128</v>
       </c>
-      <c r="K56" t="s">
-        <v>18</v>
-      </c>
-      <c r="L56" t="s">
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
         <v>129</v>
-      </c>
-    </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
-        <v>130</v>
       </c>
       <c r="B57" t="s">
         <v>13</v>
@@ -3763,12 +3760,12 @@
         <v>18</v>
       </c>
       <c r="L57" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B58" t="s">
         <v>13</v>
@@ -3814,12 +3811,12 @@
         <v>18</v>
       </c>
       <c r="L58" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B59" t="s">
         <v>13</v>
@@ -3834,10 +3831,10 @@
         <v>14</v>
       </c>
       <c r="F59" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G59" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H59" t="str">
         <f>IF(
@@ -3865,12 +3862,12 @@
         <v>18</v>
       </c>
       <c r="L59" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B60" t="s">
         <v>13</v>
@@ -3885,10 +3882,10 @@
         <v>14</v>
       </c>
       <c r="F60" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G60" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H60" t="str">
         <f>IF(
@@ -3916,12 +3913,12 @@
         <v>18</v>
       </c>
       <c r="L60" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
         <v>136</v>
-      </c>
-    </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A61" t="s">
-        <v>137</v>
       </c>
       <c r="B61" t="s">
         <v>13</v>
@@ -3933,13 +3930,13 @@
         <v>15</v>
       </c>
       <c r="E61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F61" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G61" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H61" t="str">
         <f>IF(
@@ -3961,18 +3958,18 @@
         <v>19:24:37</v>
       </c>
       <c r="J61" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="K61" t="s">
         <v>18</v>
       </c>
       <c r="L61" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B62" t="s">
         <v>13</v>
@@ -3984,13 +3981,13 @@
         <v>15</v>
       </c>
       <c r="E62" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F62" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G62" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="H62" t="str">
         <f>IF(
@@ -4018,12 +4015,12 @@
         <v>18</v>
       </c>
       <c r="L62" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B63" t="s">
         <v>13</v>
@@ -4069,12 +4066,12 @@
         <v>18</v>
       </c>
       <c r="L63" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B64" t="s">
         <v>13</v>
@@ -4114,18 +4111,18 @@
         <v>0.80763888888888891</v>
       </c>
       <c r="J64" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K64" t="s">
         <v>18</v>
       </c>
       <c r="L64" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.2">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B65" t="s">
         <v>13</v>
@@ -4171,12 +4168,12 @@
         <v>18</v>
       </c>
       <c r="L65" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.2">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B66" t="s">
         <v>13</v>
@@ -4191,10 +4188,10 @@
         <v>14</v>
       </c>
       <c r="F66" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G66" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H66" t="str">
         <f>IF(
@@ -4222,12 +4219,12 @@
         <v>18</v>
       </c>
       <c r="L66" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
         <v>146</v>
-      </c>
-    </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A67" t="s">
-        <v>147</v>
       </c>
       <c r="B67" t="s">
         <v>13</v>
@@ -4236,7 +4233,7 @@
         <v>66</v>
       </c>
       <c r="D67" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E67" t="s">
         <v>15</v>
@@ -4273,12 +4270,12 @@
         <v>18</v>
       </c>
       <c r="L67" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.2">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B68" t="s">
         <v>13</v>
@@ -4290,13 +4287,13 @@
         <v>15</v>
       </c>
       <c r="E68" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F68" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G68" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H68" t="str">
         <f>IF(
@@ -4324,12 +4321,12 @@
         <v>18</v>
       </c>
       <c r="L68" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.2">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B69" t="s">
         <v>13</v>
@@ -4375,12 +4372,12 @@
         <v>18</v>
       </c>
       <c r="L69" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.2">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B70" t="s">
         <v>13</v>
@@ -4395,10 +4392,10 @@
         <v>14</v>
       </c>
       <c r="F70" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G70" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H70" t="str">
         <f>IF(
@@ -4426,12 +4423,12 @@
         <v>18</v>
       </c>
       <c r="L70" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
         <v>153</v>
-      </c>
-    </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A71" t="s">
-        <v>154</v>
       </c>
       <c r="B71" t="s">
         <v>13</v>
@@ -4440,7 +4437,7 @@
         <v>70</v>
       </c>
       <c r="D71" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E71" t="s">
         <v>15</v>
@@ -4477,12 +4474,12 @@
         <v>18</v>
       </c>
       <c r="L71" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.2">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B72" t="s">
         <v>13</v>
@@ -4494,13 +4491,13 @@
         <v>15</v>
       </c>
       <c r="E72" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F72" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G72" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H72" t="str">
         <f>IF(
@@ -4528,12 +4525,12 @@
         <v>18</v>
       </c>
       <c r="L72" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
         <v>157</v>
-      </c>
-    </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A73" t="s">
-        <v>158</v>
       </c>
       <c r="B73" t="s">
         <v>13</v>
@@ -4542,7 +4539,7 @@
         <v>72</v>
       </c>
       <c r="D73" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E73" t="s">
         <v>15</v>
@@ -4579,12 +4576,12 @@
         <v>18</v>
       </c>
       <c r="L73" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
         <v>159</v>
-      </c>
-    </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A74" t="s">
-        <v>160</v>
       </c>
       <c r="B74" t="s">
         <v>13</v>
@@ -4599,10 +4596,10 @@
         <v>20</v>
       </c>
       <c r="F74" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G74" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H74" t="str">
         <f>IF(
@@ -4624,27 +4621,27 @@
         <v>21:46:22</v>
       </c>
       <c r="J74" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K74" t="s">
         <v>18</v>
       </c>
       <c r="L74" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A75" t="s">
+      <c r="B75" t="s">
         <v>163</v>
-      </c>
-      <c r="B75" t="s">
-        <v>164</v>
       </c>
       <c r="C75">
         <v>74</v>
       </c>
       <c r="D75" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E75" t="s">
         <v>15</v>
@@ -4675,18 +4672,18 @@
         <v>0.87638888888888888</v>
       </c>
       <c r="J75" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K75" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>162</v>
+      </c>
+      <c r="B76" t="s">
         <v>163</v>
-      </c>
-      <c r="B76" t="s">
-        <v>164</v>
       </c>
       <c r="C76">
         <v>75</v>
@@ -4695,13 +4692,13 @@
         <v>15</v>
       </c>
       <c r="E76" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F76" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G76" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H76" t="str">
         <f>IF(
@@ -4729,7 +4726,7 @@
         <v>18</v>
       </c>
       <c r="L76" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
   </sheetData>
@@ -4740,33 +4737,33 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>169</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>170</v>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C2" s="1">
         <v>0.34652777777777782</v>
@@ -4775,12 +4772,12 @@
         <v>45262</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C3" s="1">
         <v>0.34861111111111109</v>
@@ -4789,12 +4786,12 @@
         <v>45262</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C4" s="1">
         <v>0.36805555555555558</v>
@@ -4803,12 +4800,12 @@
         <v>45262</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B5" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C5" s="1">
         <v>0.37638888888888888</v>
@@ -4817,12 +4814,12 @@
         <v>45262</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C6" s="1">
         <v>0.38750000000000001</v>
@@ -4831,12 +4828,12 @@
         <v>45262</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>173</v>
+      </c>
+      <c r="B7" t="s">
         <v>174</v>
-      </c>
-      <c r="B7" t="s">
-        <v>175</v>
       </c>
       <c r="C7" s="1">
         <v>0.39305555555555549</v>
@@ -4845,12 +4842,12 @@
         <v>45262</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B8" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C8" s="1">
         <v>0.39444444444444438</v>
@@ -4859,12 +4856,12 @@
         <v>45262</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B9" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C9" s="1">
         <v>0.48888888888888887</v>
@@ -4873,12 +4870,12 @@
         <v>45262</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B10" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C10" s="1">
         <v>0.49305555555555558</v>
@@ -4887,12 +4884,12 @@
         <v>45262</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B11" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C11" s="1">
         <v>0.62013888888888891</v>
@@ -4901,12 +4898,12 @@
         <v>45262</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B12" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C12" s="1">
         <v>0.64027777777777772</v>
@@ -4915,12 +4912,12 @@
         <v>45262</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B13" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C13" s="1">
         <v>0.64166666666666672</v>
@@ -4929,12 +4926,12 @@
         <v>45262</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B14" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C14" s="1">
         <v>0.66111111111111109</v>
@@ -4943,12 +4940,12 @@
         <v>45262</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B15" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C15" s="1">
         <v>0.79305555555555551</v>
@@ -4957,12 +4954,12 @@
         <v>45262</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B16" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C16" s="1">
         <v>0.8041666666666667</v>
@@ -4971,12 +4968,12 @@
         <v>45262</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B17" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C17" s="1">
         <v>0.80902777777777779</v>
@@ -4985,12 +4982,12 @@
         <v>45262</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B18" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C18" s="1">
         <v>0.82222222222222219</v>
@@ -4999,12 +4996,12 @@
         <v>45262</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B19" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C19" s="1">
         <v>0.84444444444444444</v>
@@ -5013,12 +5010,12 @@
         <v>45262</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B20" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C20" s="1">
         <v>0.90694444444444444</v>
@@ -5027,12 +5024,12 @@
         <v>45262</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B21" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C21" s="1">
         <v>0.94166666666666665</v>

</xml_diff>